<commit_message>
feat: add plugin API, schema file support, streaming, and fluent schema builder
</commit_message>
<xml_diff>
--- a/examples/node/output/users.xlsx
+++ b/examples/node/output/users.xlsx
@@ -34,337 +34,337 @@
     <t>Country</t>
   </si>
   <si>
+    <t>mouser</t>
+  </si>
+  <si>
+    <t>as</t>
+  </si>
+  <si>
+    <t>capsize</t>
+  </si>
+  <si>
+    <t>mobilise</t>
+  </si>
+  <si>
+    <t>remand</t>
+  </si>
+  <si>
+    <t>hoof</t>
+  </si>
+  <si>
+    <t>allocation</t>
+  </si>
+  <si>
+    <t>solicit</t>
+  </si>
+  <si>
+    <t>provided</t>
+  </si>
+  <si>
+    <t>patroller</t>
+  </si>
+  <si>
+    <t>understanding</t>
+  </si>
+  <si>
+    <t>pure</t>
+  </si>
+  <si>
+    <t>that</t>
+  </si>
+  <si>
+    <t>restfully</t>
+  </si>
+  <si>
+    <t>aha</t>
+  </si>
+  <si>
+    <t>unique</t>
+  </si>
+  <si>
+    <t>fooey</t>
+  </si>
+  <si>
+    <t>pulse</t>
+  </si>
+  <si>
+    <t>what</t>
+  </si>
+  <si>
+    <t>coolly</t>
+  </si>
+  <si>
+    <t>cinema</t>
+  </si>
+  <si>
+    <t>ha</t>
+  </si>
+  <si>
+    <t>duh</t>
+  </si>
+  <si>
+    <t>unlike</t>
+  </si>
+  <si>
+    <t>design</t>
+  </si>
+  <si>
+    <t>but</t>
+  </si>
+  <si>
+    <t>whoever</t>
+  </si>
+  <si>
+    <t>unless</t>
+  </si>
+  <si>
+    <t>despite</t>
+  </si>
+  <si>
+    <t>bah</t>
+  </si>
+  <si>
+    <t>unethically</t>
+  </si>
+  <si>
+    <t>catalyze</t>
+  </si>
+  <si>
+    <t>idealistic</t>
+  </si>
+  <si>
+    <t>ligate</t>
+  </si>
+  <si>
+    <t>mentor</t>
+  </si>
+  <si>
+    <t>plumber</t>
+  </si>
+  <si>
+    <t>abnormally</t>
+  </si>
+  <si>
+    <t>privilege</t>
+  </si>
+  <si>
+    <t>than</t>
+  </si>
+  <si>
+    <t>cosset</t>
+  </si>
+  <si>
+    <t>actual</t>
+  </si>
+  <si>
+    <t>intently</t>
+  </si>
+  <si>
+    <t>drat</t>
+  </si>
+  <si>
+    <t>mmm</t>
+  </si>
+  <si>
+    <t>anti</t>
+  </si>
+  <si>
+    <t>mozzarella</t>
+  </si>
+  <si>
+    <t>young</t>
+  </si>
+  <si>
+    <t>or</t>
+  </si>
+  <si>
+    <t>hole</t>
+  </si>
+  <si>
+    <t>faraway</t>
+  </si>
+  <si>
+    <t>about</t>
+  </si>
+  <si>
+    <t>preregister</t>
+  </si>
+  <si>
+    <t>except</t>
+  </si>
+  <si>
+    <t>briskly</t>
+  </si>
+  <si>
+    <t>arrogantly</t>
+  </si>
+  <si>
+    <t>soulful</t>
+  </si>
+  <si>
+    <t>whistle</t>
+  </si>
+  <si>
+    <t>appropriate</t>
+  </si>
+  <si>
+    <t>crossly</t>
+  </si>
+  <si>
+    <t>gee</t>
+  </si>
+  <si>
+    <t>bookcase</t>
+  </si>
+  <si>
     <t>for</t>
   </si>
   <si>
+    <t>finally</t>
+  </si>
+  <si>
+    <t>antique</t>
+  </si>
+  <si>
+    <t>ugh</t>
+  </si>
+  <si>
+    <t>yippee</t>
+  </si>
+  <si>
+    <t>blah</t>
+  </si>
+  <si>
+    <t>nor</t>
+  </si>
+  <si>
+    <t>entry</t>
+  </si>
+  <si>
+    <t>rubbery</t>
+  </si>
+  <si>
+    <t>flood</t>
+  </si>
+  <si>
+    <t>yesterday</t>
+  </si>
+  <si>
+    <t>pfft</t>
+  </si>
+  <si>
+    <t>oh</t>
+  </si>
+  <si>
+    <t>phrase</t>
+  </si>
+  <si>
+    <t>suitcase</t>
+  </si>
+  <si>
+    <t>squirm</t>
+  </si>
+  <si>
+    <t>dimly</t>
+  </si>
+  <si>
+    <t>whoa</t>
+  </si>
+  <si>
+    <t>lightly</t>
+  </si>
+  <si>
+    <t>instead</t>
+  </si>
+  <si>
+    <t>midst</t>
+  </si>
+  <si>
+    <t>with</t>
+  </si>
+  <si>
+    <t>edge</t>
+  </si>
+  <si>
+    <t>until</t>
+  </si>
+  <si>
+    <t>flight</t>
+  </si>
+  <si>
+    <t>electronics</t>
+  </si>
+  <si>
+    <t>christen</t>
+  </si>
+  <si>
+    <t>sweetly</t>
+  </si>
+  <si>
+    <t>generously</t>
+  </si>
+  <si>
+    <t>huzzah</t>
+  </si>
+  <si>
+    <t>marksman</t>
+  </si>
+  <si>
+    <t>never</t>
+  </si>
+  <si>
+    <t>careless</t>
+  </si>
+  <si>
+    <t>reschedule</t>
+  </si>
+  <si>
+    <t>er</t>
+  </si>
+  <si>
+    <t>uproot</t>
+  </si>
+  <si>
+    <t>harmful</t>
+  </si>
+  <si>
+    <t>against</t>
+  </si>
+  <si>
+    <t>likewise</t>
+  </si>
+  <si>
+    <t>before</t>
+  </si>
+  <si>
+    <t>versus</t>
+  </si>
+  <si>
+    <t>yuck</t>
+  </si>
+  <si>
+    <t>order</t>
+  </si>
+  <si>
+    <t>triumphantly</t>
+  </si>
+  <si>
     <t>while</t>
   </si>
   <si>
-    <t>antique</t>
-  </si>
-  <si>
-    <t>truthfully</t>
-  </si>
-  <si>
-    <t>tackle</t>
-  </si>
-  <si>
-    <t>wearily</t>
-  </si>
-  <si>
-    <t>indeed</t>
-  </si>
-  <si>
-    <t>against</t>
-  </si>
-  <si>
-    <t>decriminalize</t>
-  </si>
-  <si>
-    <t>whoever</t>
-  </si>
-  <si>
-    <t>creaking</t>
-  </si>
-  <si>
-    <t>monster</t>
-  </si>
-  <si>
-    <t>whirlwind</t>
-  </si>
-  <si>
-    <t>gee</t>
-  </si>
-  <si>
-    <t>along</t>
-  </si>
-  <si>
-    <t>successfully</t>
-  </si>
-  <si>
-    <t>hype</t>
-  </si>
-  <si>
-    <t>twine</t>
-  </si>
-  <si>
-    <t>critical</t>
-  </si>
-  <si>
-    <t>drat</t>
-  </si>
-  <si>
-    <t>calculus</t>
-  </si>
-  <si>
-    <t>ah</t>
-  </si>
-  <si>
-    <t>whose</t>
-  </si>
-  <si>
-    <t>aircraft</t>
-  </si>
-  <si>
-    <t>clonk</t>
-  </si>
-  <si>
-    <t>consequently</t>
-  </si>
-  <si>
-    <t>quirkily</t>
-  </si>
-  <si>
-    <t>nor</t>
-  </si>
-  <si>
-    <t>er</t>
-  </si>
-  <si>
-    <t>lovingly</t>
-  </si>
-  <si>
-    <t>collaboration</t>
-  </si>
-  <si>
-    <t>positively</t>
-  </si>
-  <si>
-    <t>however</t>
-  </si>
-  <si>
-    <t>into</t>
-  </si>
-  <si>
-    <t>finally</t>
-  </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>sit</t>
-  </si>
-  <si>
-    <t>longingly</t>
-  </si>
-  <si>
-    <t>eyeglasses</t>
-  </si>
-  <si>
-    <t>junior</t>
-  </si>
-  <si>
-    <t>reckon</t>
-  </si>
-  <si>
-    <t>times</t>
-  </si>
-  <si>
-    <t>after</t>
-  </si>
-  <si>
-    <t>during</t>
-  </si>
-  <si>
-    <t>between</t>
-  </si>
-  <si>
-    <t>emphasise</t>
-  </si>
-  <si>
-    <t>dicker</t>
-  </si>
-  <si>
-    <t>hm</t>
-  </si>
-  <si>
-    <t>aside</t>
-  </si>
-  <si>
-    <t>spectate</t>
-  </si>
-  <si>
-    <t>paltry</t>
-  </si>
-  <si>
-    <t>indolent</t>
-  </si>
-  <si>
-    <t>wry</t>
-  </si>
-  <si>
-    <t>packaging</t>
-  </si>
-  <si>
-    <t>simplistic</t>
-  </si>
-  <si>
-    <t>resort</t>
-  </si>
-  <si>
-    <t>glorious</t>
-  </si>
-  <si>
-    <t>round</t>
-  </si>
-  <si>
-    <t>step</t>
-  </si>
-  <si>
-    <t>hmph</t>
-  </si>
-  <si>
-    <t>excepting</t>
-  </si>
-  <si>
-    <t>yuck</t>
-  </si>
-  <si>
-    <t>phew</t>
-  </si>
-  <si>
-    <t>exterior</t>
-  </si>
-  <si>
-    <t>peppery</t>
-  </si>
-  <si>
-    <t>amongst</t>
-  </si>
-  <si>
-    <t>blowgun</t>
-  </si>
-  <si>
-    <t>wilted</t>
-  </si>
-  <si>
-    <t>chromakey</t>
-  </si>
-  <si>
-    <t>failing</t>
-  </si>
-  <si>
-    <t>quicker</t>
-  </si>
-  <si>
-    <t>pace</t>
-  </si>
-  <si>
-    <t>ick</t>
-  </si>
-  <si>
-    <t>puritan</t>
-  </si>
-  <si>
-    <t>circa</t>
-  </si>
-  <si>
-    <t>sediment</t>
-  </si>
-  <si>
-    <t>mmm</t>
-  </si>
-  <si>
-    <t>how</t>
-  </si>
-  <si>
-    <t>superficial</t>
-  </si>
-  <si>
-    <t>colorful</t>
-  </si>
-  <si>
-    <t>yet</t>
-  </si>
-  <si>
-    <t>pick</t>
-  </si>
-  <si>
-    <t>without</t>
-  </si>
-  <si>
-    <t>filter</t>
-  </si>
-  <si>
-    <t>though</t>
-  </si>
-  <si>
-    <t>till</t>
-  </si>
-  <si>
-    <t>video</t>
-  </si>
-  <si>
-    <t>internationalize</t>
-  </si>
-  <si>
-    <t>vet</t>
-  </si>
-  <si>
-    <t>lady</t>
-  </si>
-  <si>
-    <t>notwithstanding</t>
-  </si>
-  <si>
-    <t>ugh</t>
-  </si>
-  <si>
-    <t>chairperson</t>
-  </si>
-  <si>
-    <t>optimistic</t>
-  </si>
-  <si>
-    <t>judicious</t>
-  </si>
-  <si>
-    <t>uh-huh</t>
-  </si>
-  <si>
-    <t>jell</t>
-  </si>
-  <si>
-    <t>gadzooks</t>
-  </si>
-  <si>
-    <t>if</t>
-  </si>
-  <si>
-    <t>traffic</t>
-  </si>
-  <si>
-    <t>disk</t>
-  </si>
-  <si>
-    <t>before</t>
-  </si>
-  <si>
-    <t>seldom</t>
-  </si>
-  <si>
-    <t>instead</t>
-  </si>
-  <si>
-    <t>sweet</t>
-  </si>
-  <si>
-    <t>furthermore</t>
-  </si>
-  <si>
-    <t>or</t>
-  </si>
-  <si>
-    <t>platter</t>
-  </si>
-  <si>
-    <t>happily</t>
-  </si>
-  <si>
-    <t>monasticism</t>
-  </si>
-  <si>
-    <t>harp</t>
+    <t>broadcast</t>
+  </si>
+  <si>
+    <t>scenario</t>
+  </si>
+  <si>
+    <t>zebra</t>
+  </si>
+  <si>
+    <t>vision</t>
+  </si>
+  <si>
+    <t>spirit</t>
   </si>
 </sst>
 </file>
@@ -754,12 +754,11 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="4" width="13" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -868,13 +867,13 @@
         <v>27</v>
       </c>
       <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
         <v>28</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>29</v>
-      </c>
-      <c r="G5" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -882,22 +881,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
         <v>31</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>32</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>33</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>34</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>35</v>
-      </c>
-      <c r="G6" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -905,13 +904,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
         <v>37</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>38</v>
-      </c>
-      <c r="D7" t="s">
-        <v>13</v>
       </c>
       <c r="E7" t="s">
         <v>39</v>
@@ -934,16 +933,16 @@
         <v>43</v>
       </c>
       <c r="D8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" t="s">
         <v>44</v>
       </c>
-      <c r="E8" t="s">
+      <c r="F8" t="s">
         <v>45</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>46</v>
-      </c>
-      <c r="G8" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -951,22 +950,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" t="s">
         <v>48</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>49</v>
       </c>
-      <c r="D9" t="s">
-        <v>50</v>
-      </c>
       <c r="E9" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="G9" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,22 +973,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C10" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" t="s">
         <v>54</v>
       </c>
-      <c r="C10" t="s">
+      <c r="G10" t="s">
         <v>55</v>
-      </c>
-      <c r="D10" t="s">
-        <v>56</v>
-      </c>
-      <c r="E10" t="s">
-        <v>57</v>
-      </c>
-      <c r="F10" t="s">
-        <v>58</v>
-      </c>
-      <c r="G10" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -997,22 +996,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" t="s">
         <v>60</v>
       </c>
-      <c r="C11" t="s">
+      <c r="G11" t="s">
         <v>61</v>
-      </c>
-      <c r="D11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E11" t="s">
-        <v>62</v>
-      </c>
-      <c r="F11" t="s">
-        <v>63</v>
-      </c>
-      <c r="G11" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1020,22 +1019,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" t="s">
+        <v>64</v>
+      </c>
+      <c r="E12" t="s">
         <v>65</v>
       </c>
-      <c r="C12" t="s">
+      <c r="F12" t="s">
         <v>66</v>
       </c>
-      <c r="D12" t="s">
+      <c r="G12" t="s">
         <v>67</v>
-      </c>
-      <c r="E12" t="s">
-        <v>68</v>
-      </c>
-      <c r="F12" t="s">
-        <v>69</v>
-      </c>
-      <c r="G12" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1043,22 +1042,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13" t="s">
         <v>71</v>
       </c>
-      <c r="C13" t="s">
+      <c r="F13" t="s">
+        <v>33</v>
+      </c>
+      <c r="G13" t="s">
         <v>72</v>
-      </c>
-      <c r="D13" t="s">
-        <v>73</v>
-      </c>
-      <c r="E13" t="s">
-        <v>74</v>
-      </c>
-      <c r="F13" t="s">
-        <v>75</v>
-      </c>
-      <c r="G13" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1066,22 +1065,22 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
+        <v>73</v>
+      </c>
+      <c r="C14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" t="s">
+        <v>75</v>
+      </c>
+      <c r="E14" t="s">
+        <v>76</v>
+      </c>
+      <c r="F14" t="s">
         <v>77</v>
       </c>
-      <c r="C14" t="s">
+      <c r="G14" t="s">
         <v>78</v>
-      </c>
-      <c r="D14" t="s">
-        <v>79</v>
-      </c>
-      <c r="E14" t="s">
-        <v>80</v>
-      </c>
-      <c r="F14" t="s">
-        <v>81</v>
-      </c>
-      <c r="G14" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1089,22 +1088,22 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E15" t="s">
         <v>82</v>
       </c>
-      <c r="C15" t="s">
+      <c r="F15" t="s">
         <v>83</v>
       </c>
-      <c r="D15" t="s">
+      <c r="G15" t="s">
         <v>84</v>
-      </c>
-      <c r="E15" t="s">
-        <v>85</v>
-      </c>
-      <c r="F15" t="s">
-        <v>86</v>
-      </c>
-      <c r="G15" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1112,22 +1111,22 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>49</v>
+        <v>85</v>
       </c>
       <c r="C16" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" t="s">
+        <v>87</v>
+      </c>
+      <c r="E16" t="s">
         <v>88</v>
       </c>
-      <c r="D16" t="s">
+      <c r="F16" t="s">
         <v>89</v>
       </c>
-      <c r="E16" t="s">
+      <c r="G16" t="s">
         <v>90</v>
-      </c>
-      <c r="F16" t="s">
-        <v>91</v>
-      </c>
-      <c r="G16" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1135,22 +1134,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" t="s">
         <v>93</v>
       </c>
-      <c r="C17" t="s">
+      <c r="E17" t="s">
         <v>94</v>
       </c>
-      <c r="D17" t="s">
+      <c r="F17" t="s">
         <v>95</v>
       </c>
-      <c r="E17" t="s">
+      <c r="G17" t="s">
         <v>96</v>
-      </c>
-      <c r="F17" t="s">
-        <v>97</v>
-      </c>
-      <c r="G17" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1158,22 +1157,22 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C18" t="s">
+        <v>98</v>
+      </c>
+      <c r="D18" t="s">
         <v>99</v>
       </c>
-      <c r="C18" t="s">
+      <c r="E18" t="s">
         <v>100</v>
       </c>
-      <c r="D18" t="s">
+      <c r="F18" t="s">
         <v>101</v>
       </c>
-      <c r="E18" t="s">
-        <v>87</v>
-      </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>102</v>
-      </c>
-      <c r="G18" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1181,22 +1180,22 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>74</v>
       </c>
       <c r="C19" t="s">
+        <v>103</v>
+      </c>
+      <c r="D19" t="s">
         <v>104</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>105</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>106</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>107</v>
-      </c>
-      <c r="G19" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1204,22 +1203,22 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>66</v>
+        <v>108</v>
       </c>
       <c r="C20" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D20" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E20" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="F20" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G20" t="s">
-        <v>68</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1227,13 +1226,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C21" t="s">
-        <v>113</v>
+        <v>72</v>
       </c>
       <c r="D21" t="s">
-        <v>114</v>
+        <v>71</v>
       </c>
       <c r="E21" t="s">
         <v>115</v>

</xml_diff>

<commit_message>
feat: add schema inference, OpenAPI/GraphQL bridges, watch mode, Parquet support, streaming API, and schema builder UI
</commit_message>
<xml_diff>
--- a/examples/node/output/users.xlsx
+++ b/examples/node/output/users.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="119">
   <si>
     <t>Id</t>
   </si>
@@ -34,337 +34,340 @@
     <t>Country</t>
   </si>
   <si>
-    <t>mouser</t>
-  </si>
-  <si>
-    <t>as</t>
-  </si>
-  <si>
-    <t>capsize</t>
-  </si>
-  <si>
-    <t>mobilise</t>
-  </si>
-  <si>
-    <t>remand</t>
-  </si>
-  <si>
-    <t>hoof</t>
-  </si>
-  <si>
-    <t>allocation</t>
-  </si>
-  <si>
-    <t>solicit</t>
-  </si>
-  <si>
-    <t>provided</t>
-  </si>
-  <si>
-    <t>patroller</t>
+    <t>failing</t>
   </si>
   <si>
     <t>understanding</t>
   </si>
   <si>
-    <t>pure</t>
-  </si>
-  <si>
-    <t>that</t>
-  </si>
-  <si>
-    <t>restfully</t>
+    <t>promptly</t>
+  </si>
+  <si>
+    <t>silver</t>
+  </si>
+  <si>
+    <t>dual</t>
+  </si>
+  <si>
+    <t>times</t>
+  </si>
+  <si>
+    <t>er</t>
+  </si>
+  <si>
+    <t>poorly</t>
+  </si>
+  <si>
+    <t>punctuation</t>
+  </si>
+  <si>
+    <t>including</t>
+  </si>
+  <si>
+    <t>limply</t>
+  </si>
+  <si>
+    <t>meanwhile</t>
+  </si>
+  <si>
+    <t>wing</t>
+  </si>
+  <si>
+    <t>oh</t>
+  </si>
+  <si>
+    <t>accidentally</t>
+  </si>
+  <si>
+    <t>dusk</t>
+  </si>
+  <si>
+    <t>duh</t>
+  </si>
+  <si>
+    <t>across</t>
+  </si>
+  <si>
+    <t>mentor</t>
+  </si>
+  <si>
+    <t>braid</t>
+  </si>
+  <si>
+    <t>joyfully</t>
+  </si>
+  <si>
+    <t>courageously</t>
+  </si>
+  <si>
+    <t>deflate</t>
+  </si>
+  <si>
+    <t>instead</t>
+  </si>
+  <si>
+    <t>dental</t>
+  </si>
+  <si>
+    <t>geez</t>
+  </si>
+  <si>
+    <t>outgoing</t>
+  </si>
+  <si>
+    <t>brush</t>
+  </si>
+  <si>
+    <t>homely</t>
+  </si>
+  <si>
+    <t>opposite</t>
+  </si>
+  <si>
+    <t>institutionalize</t>
+  </si>
+  <si>
+    <t>burly</t>
+  </si>
+  <si>
+    <t>unless</t>
+  </si>
+  <si>
+    <t>squirm</t>
+  </si>
+  <si>
+    <t>pro</t>
+  </si>
+  <si>
+    <t>and</t>
+  </si>
+  <si>
+    <t>parsnip</t>
+  </si>
+  <si>
+    <t>yowza</t>
+  </si>
+  <si>
+    <t>spanish</t>
+  </si>
+  <si>
+    <t>trek</t>
+  </si>
+  <si>
+    <t>shallow</t>
+  </si>
+  <si>
+    <t>subdued</t>
+  </si>
+  <si>
+    <t>coal</t>
+  </si>
+  <si>
+    <t>before</t>
+  </si>
+  <si>
+    <t>simple</t>
+  </si>
+  <si>
+    <t>cow</t>
+  </si>
+  <si>
+    <t>noisily</t>
+  </si>
+  <si>
+    <t>dishearten</t>
+  </si>
+  <si>
+    <t>home</t>
   </si>
   <si>
     <t>aha</t>
   </si>
   <si>
-    <t>unique</t>
-  </si>
-  <si>
-    <t>fooey</t>
-  </si>
-  <si>
-    <t>pulse</t>
+    <t>than</t>
+  </si>
+  <si>
+    <t>chilly</t>
+  </si>
+  <si>
+    <t>acclaimed</t>
+  </si>
+  <si>
+    <t>weep</t>
+  </si>
+  <si>
+    <t>continually</t>
+  </si>
+  <si>
+    <t>honestly</t>
+  </si>
+  <si>
+    <t>frank</t>
+  </si>
+  <si>
+    <t>kiss</t>
+  </si>
+  <si>
+    <t>bicycle</t>
+  </si>
+  <si>
+    <t>coliseum</t>
+  </si>
+  <si>
+    <t>cauliflower</t>
+  </si>
+  <si>
+    <t>hold</t>
+  </si>
+  <si>
+    <t>octave</t>
+  </si>
+  <si>
+    <t>limited</t>
+  </si>
+  <si>
+    <t>huzzah</t>
+  </si>
+  <si>
+    <t>angelic</t>
+  </si>
+  <si>
+    <t>apricot</t>
+  </si>
+  <si>
+    <t>casement</t>
+  </si>
+  <si>
+    <t>boldly</t>
+  </si>
+  <si>
+    <t>gosh</t>
+  </si>
+  <si>
+    <t>midst</t>
+  </si>
+  <si>
+    <t>unabashedly</t>
+  </si>
+  <si>
+    <t>but</t>
+  </si>
+  <si>
+    <t>unblinking</t>
+  </si>
+  <si>
+    <t>culminate</t>
+  </si>
+  <si>
+    <t>wring</t>
   </si>
   <si>
     <t>what</t>
   </si>
   <si>
-    <t>coolly</t>
-  </si>
-  <si>
-    <t>cinema</t>
-  </si>
-  <si>
-    <t>ha</t>
-  </si>
-  <si>
-    <t>duh</t>
-  </si>
-  <si>
-    <t>unlike</t>
-  </si>
-  <si>
-    <t>design</t>
-  </si>
-  <si>
-    <t>but</t>
-  </si>
-  <si>
-    <t>whoever</t>
-  </si>
-  <si>
-    <t>unless</t>
-  </si>
-  <si>
-    <t>despite</t>
-  </si>
-  <si>
-    <t>bah</t>
-  </si>
-  <si>
-    <t>unethically</t>
-  </si>
-  <si>
-    <t>catalyze</t>
-  </si>
-  <si>
-    <t>idealistic</t>
-  </si>
-  <si>
-    <t>ligate</t>
-  </si>
-  <si>
-    <t>mentor</t>
-  </si>
-  <si>
-    <t>plumber</t>
-  </si>
-  <si>
-    <t>abnormally</t>
-  </si>
-  <si>
-    <t>privilege</t>
-  </si>
-  <si>
-    <t>than</t>
-  </si>
-  <si>
-    <t>cosset</t>
-  </si>
-  <si>
-    <t>actual</t>
-  </si>
-  <si>
-    <t>intently</t>
-  </si>
-  <si>
-    <t>drat</t>
-  </si>
-  <si>
-    <t>mmm</t>
-  </si>
-  <si>
-    <t>anti</t>
-  </si>
-  <si>
-    <t>mozzarella</t>
-  </si>
-  <si>
-    <t>young</t>
-  </si>
-  <si>
-    <t>or</t>
-  </si>
-  <si>
-    <t>hole</t>
-  </si>
-  <si>
-    <t>faraway</t>
-  </si>
-  <si>
-    <t>about</t>
-  </si>
-  <si>
-    <t>preregister</t>
-  </si>
-  <si>
-    <t>except</t>
-  </si>
-  <si>
-    <t>briskly</t>
-  </si>
-  <si>
-    <t>arrogantly</t>
-  </si>
-  <si>
-    <t>soulful</t>
-  </si>
-  <si>
-    <t>whistle</t>
-  </si>
-  <si>
-    <t>appropriate</t>
-  </si>
-  <si>
-    <t>crossly</t>
+    <t>clamour</t>
+  </si>
+  <si>
+    <t>ack</t>
+  </si>
+  <si>
+    <t>oddly</t>
+  </si>
+  <si>
+    <t>candid</t>
+  </si>
+  <si>
+    <t>scarcely</t>
+  </si>
+  <si>
+    <t>plus</t>
+  </si>
+  <si>
+    <t>mindless</t>
+  </si>
+  <si>
+    <t>junior</t>
+  </si>
+  <si>
+    <t>corner</t>
+  </si>
+  <si>
+    <t>once</t>
+  </si>
+  <si>
+    <t>actually</t>
+  </si>
+  <si>
+    <t>fatally</t>
+  </si>
+  <si>
+    <t>bourgeoisie</t>
+  </si>
+  <si>
+    <t>after</t>
+  </si>
+  <si>
+    <t>nor</t>
+  </si>
+  <si>
+    <t>shrilly</t>
+  </si>
+  <si>
+    <t>gratefully</t>
+  </si>
+  <si>
+    <t>who</t>
+  </si>
+  <si>
+    <t>soap</t>
+  </si>
+  <si>
+    <t>although</t>
+  </si>
+  <si>
+    <t>jealously</t>
+  </si>
+  <si>
+    <t>deficient</t>
+  </si>
+  <si>
+    <t>seemingly</t>
+  </si>
+  <si>
+    <t>excitedly</t>
+  </si>
+  <si>
+    <t>shabby</t>
   </si>
   <si>
     <t>gee</t>
   </si>
   <si>
-    <t>bookcase</t>
-  </si>
-  <si>
-    <t>for</t>
-  </si>
-  <si>
-    <t>finally</t>
-  </si>
-  <si>
-    <t>antique</t>
-  </si>
-  <si>
-    <t>ugh</t>
-  </si>
-  <si>
-    <t>yippee</t>
-  </si>
-  <si>
-    <t>blah</t>
-  </si>
-  <si>
-    <t>nor</t>
-  </si>
-  <si>
-    <t>entry</t>
-  </si>
-  <si>
-    <t>rubbery</t>
-  </si>
-  <si>
-    <t>flood</t>
-  </si>
-  <si>
-    <t>yesterday</t>
-  </si>
-  <si>
-    <t>pfft</t>
-  </si>
-  <si>
-    <t>oh</t>
-  </si>
-  <si>
-    <t>phrase</t>
-  </si>
-  <si>
-    <t>suitcase</t>
-  </si>
-  <si>
-    <t>squirm</t>
-  </si>
-  <si>
-    <t>dimly</t>
-  </si>
-  <si>
-    <t>whoa</t>
-  </si>
-  <si>
-    <t>lightly</t>
-  </si>
-  <si>
-    <t>instead</t>
-  </si>
-  <si>
-    <t>midst</t>
-  </si>
-  <si>
-    <t>with</t>
-  </si>
-  <si>
-    <t>edge</t>
-  </si>
-  <si>
-    <t>until</t>
-  </si>
-  <si>
-    <t>flight</t>
-  </si>
-  <si>
-    <t>electronics</t>
-  </si>
-  <si>
-    <t>christen</t>
-  </si>
-  <si>
-    <t>sweetly</t>
-  </si>
-  <si>
-    <t>generously</t>
-  </si>
-  <si>
-    <t>huzzah</t>
-  </si>
-  <si>
-    <t>marksman</t>
-  </si>
-  <si>
-    <t>never</t>
-  </si>
-  <si>
-    <t>careless</t>
-  </si>
-  <si>
-    <t>reschedule</t>
-  </si>
-  <si>
-    <t>er</t>
-  </si>
-  <si>
-    <t>uproot</t>
-  </si>
-  <si>
-    <t>harmful</t>
-  </si>
-  <si>
-    <t>against</t>
-  </si>
-  <si>
-    <t>likewise</t>
-  </si>
-  <si>
-    <t>before</t>
-  </si>
-  <si>
-    <t>versus</t>
-  </si>
-  <si>
-    <t>yuck</t>
-  </si>
-  <si>
-    <t>order</t>
-  </si>
-  <si>
-    <t>triumphantly</t>
-  </si>
-  <si>
-    <t>while</t>
-  </si>
-  <si>
-    <t>broadcast</t>
-  </si>
-  <si>
-    <t>scenario</t>
-  </si>
-  <si>
-    <t>zebra</t>
-  </si>
-  <si>
-    <t>vision</t>
-  </si>
-  <si>
-    <t>spirit</t>
+    <t>pulverize</t>
+  </si>
+  <si>
+    <t>uselessly</t>
+  </si>
+  <si>
+    <t>warmhearted</t>
+  </si>
+  <si>
+    <t>phooey</t>
+  </si>
+  <si>
+    <t>numb</t>
+  </si>
+  <si>
+    <t>cheerfully</t>
+  </si>
+  <si>
+    <t>slake</t>
+  </si>
+  <si>
+    <t>under</t>
+  </si>
+  <si>
+    <t>awkwardly</t>
   </si>
 </sst>
 </file>
@@ -754,10 +757,10 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
@@ -867,13 +870,13 @@
         <v>27</v>
       </c>
       <c r="E5" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -881,22 +884,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -904,22 +907,22 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -927,22 +930,22 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D8" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="E8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -950,22 +953,22 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E9" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="F9" t="s">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="G9" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -973,22 +976,22 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="E10" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G10" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -996,22 +999,22 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G11" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -1019,22 +1022,22 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="D12" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="E12" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G12" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -1042,22 +1045,22 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="D13" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E13" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F13" t="s">
-        <v>33</v>
+        <v>75</v>
       </c>
       <c r="G13" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -1065,22 +1068,22 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C14" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D14" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F14" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G14" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -1088,22 +1091,22 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C15" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D15" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="E15" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="F15" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="G15" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1111,22 +1114,22 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C16" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D16" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E16" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F16" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G16" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1134,22 +1137,22 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C17" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D17" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="E17" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F17" t="s">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="G17" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1157,22 +1160,22 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C18" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D18" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E18" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F18" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="G18" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1180,22 +1183,22 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>106</v>
       </c>
       <c r="C19" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D19" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="E19" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="F19" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="G19" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1203,22 +1206,22 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C20" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D20" t="s">
-        <v>110</v>
+        <v>61</v>
       </c>
       <c r="E20" t="s">
-        <v>111</v>
+        <v>30</v>
       </c>
       <c r="F20" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G20" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1226,22 +1229,22 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C21" t="s">
-        <v>72</v>
+        <v>116</v>
       </c>
       <c r="D21" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="E21" t="s">
-        <v>115</v>
+        <v>56</v>
       </c>
       <c r="F21" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G21" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>